<commit_message>
Tie-in register: structured tie-in conditions, tie_in_register engine, agreement rounds
- tie_in schema: category, scope break, connection, isolation, protection, operating
  envelope (barg/degC), capacity, electrical data, HMB stream/metric, upstream chain,
  dates, agreement (status, agreed_by, agreed_ref)
- tie_in_register engine (xlsx + docx + pdf) with checks: completeness, HMB envelope
  over all 9 cases, Owner-EPC-IEC chain, dates, agreement, scope coverage; tests
- TQ-IEC-021: ST valve casing design, new IF-45/IF-46 (spray water), IF-03 location,
  IPB tap-off rating; IEC-ALP-IF-001 Rev A registered; all IF points agreed
- TQ-030..032 and TQ-027 answered by the Owner: TP-A2, TP-T2, TP-T3 added, missing data
  supplied, export limiter 640 MW; all TP points agreed
- lesson L-EPCE-0001

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TuQPCZMPzEzscTVqEEHFMo
</commit_message>
<xml_diff>
--- a/output/clarification_register/ALP_clarification_register_ALP-CA-001.xlsx
+++ b/output/clarification_register/ALP_clarification_register_ALP-CA-001.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -481,7 +481,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>engine clarification_register v1.1.0 | generated 2026-09-28T03:17:00Z by SETUP | data 697afb309489c934</t>
+          <t>engine clarification_register v1.1.0 | generated 2026-09-28T03:43:27Z by SETUP | data 739c56375ca05fc7</t>
         </is>
       </c>
     </row>
@@ -2196,6 +2196,137 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>TQ-IEC-021</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Istanbul EPC</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Tie-in register: interface conditions IF-01..IF-44 for agreement</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>The EPC tie-in register (engine tie_in_register, draft) checks every terminal point against the nine PER-003 Rev A cases and against its upstream point. Please confirm or correct: (1) IF-06 (200 bar(a) / 605 degC), IF-10 (48 bar(a) / 605 degC) and IF-12 (8 bar(a)) are below the design of the HRSG outlets feeding them (IF-05 210 bar(a) / 610 degC, IF-09 50 bar(a) / 610 degC, IF-11 10 bar(a)); the EPC piping between them is designed for the HRSG side. State the ST valve casing design conditions, or the safety valve set points that protect the ST side. (2) HMB streams 29 and 30 (HP and reheat attemperation spray water from the EPC BFP discharge/interstage to the HRSG) cross the scope boundary but have no terminal point in IF-001 Rev 0. (3) PER-003 stream 28 (water injection) is at 60 bar(a), IF-03 is 4 in CL150 / 16 barg: confirm IF-03 is at the skid inlet upstream of IEC injection pumps, the pressure required there, and that the pump power is in the IEC auxiliaries. (4) IF-36: the EPC estimates 169 kA prospective short-circuit current at the GT generator bus (96 kA from the system via the GSU + 73 kA from the generator); state the IPB tap-off rating. (5) Confirm the operating envelopes, scope breaks, isolation, protection and dates of the attached draft (dates per the EPC commissioning sequence DEC-EPCE-0004) and re-issue IF-001.</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>(1) ST valve casings designed for the HRSG outlet conditions; (2) new IF-45 / IF-46 at the inlet of the IEC spray control stations; (3) IF-03 at the skid inlet, 3.0-6.0 barg; (4) tap-off rated &gt;= 170 kA; (5) IF-001 Rev A with the agreed data.</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>tie_in:IF-03
+tie_in:IF-06
+tie_in:IF-10
+tie_in:IF-12
+tie_in:IF-36
+process_stream:SRC-LDO-100_28
+process_stream:MAX-NG-100_29
+process_stream:MAX-NG-100_30
+source:SRC-EPCE-0008
+source:SRC-IECE-0005</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>(1) The IF-001 Rev 0 values at IF-06/IF-10/IF-12 were the ST rated inlet conditions (IEC 60045-1). Valve casing design: main stop valve 215 bar(a) / 610 degC, IP stop/control valves 52 bar(a) / 610 degC, LP admission valve 10 bar(a) / 330 degC; the HRSG safety valves (HP SH &lt;= 196 bar(a), HRH &lt;= 48 bar(a), LP SH 8.0 bar(a)) protect both sides. (2) Accepted: IF-45 (HP spray, 3 in CL2500) and IF-46 (reheat spray, 2 in CL600) at the inlet of the IEC spray control stations. (3) Confirmed: IF-03 is the water injection skid inlet, 3.0-6.0 barg; stream 28 in PER-003 is the skid discharge; the injection pumps are in the IEC GT auxiliaries. (4) IPB tap-off rated 200 kA symmetrical / 550 kA peak. (5) Draft data confirmed with the corrections above; IEC-ALP-IF-001 Rev A issued.</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>contractor proposal accepted</t>
+        </is>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>technical_only</t>
+        </is>
+      </c>
+      <c r="P25" s="4" t="n"/>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>tie_in/IF-01
+tie_in/IF-02
+tie_in/IF-03
+tie_in/IF-04
+tie_in/IF-05
+tie_in/IF-06
+tie_in/IF-07
+tie_in/IF-08
+tie_in/IF-09
+tie_in/IF-10
+tie_in/IF-11
+tie_in/IF-12
+tie_in/IF-13
+tie_in/IF-14
+tie_in/IF-15
+tie_in/IF-16
+tie_in/IF-17
+tie_in/IF-18
+tie_in/IF-19
+tie_in/IF-20
+tie_in/IF-21
+tie_in/IF-22
+tie_in/IF-23
+tie_in/IF-24
+tie_in/IF-25
+tie_in/IF-26
+tie_in/IF-27
+tie_in/IF-28
+tie_in/IF-29
+tie_in/IF-30
+tie_in/IF-31
+tie_in/IF-32
+tie_in/IF-33
+tie_in/IF-34
+tie_in/IF-35
+tie_in/IF-36
+tie_in/IF-37
+tie_in/IF-38
+tie_in/IF-39
+tie_in/IF-40
+tie_in/IF-41
+tie_in/IF-42
+tie_in/IF-43
+tie_in/IF-44
+tie_in/IF-45
+tie_in/IF-46</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:Q4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2209,7 +2340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2342,77 +2473,96 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Round 6</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="D7" s="6" t="n">
+      <c r="B8" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="D8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="E8" s="6" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>By outcome</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>confirmed as is</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>8</v>
-      </c>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>contractor proposal accepted</t>
+          <t>confirmed as is</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>follow up required</t>
+          <t>contractor proposal accepted</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>follow up required</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>requirement changed</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B14" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Codes, standards and permits register (Appendix A.19) agreed with the Owner and IEC
- reference schema extended (kind, precedence, responsible, authority, requirements,
  deviation, agreement); new permit entity; 14 authority parties
- 100 register entries (Turkish laws/regulations, Grid Code, codes and standards) and
  24 permits with applicant, deliverables, lead time and need dates
- standards_register engine (xlsx + docx + pdf): ER citation coverage, authorities,
  agreement, permit timing; tests
- TQ-033 (Owner) and TQ-IEC-022 (IEC) closed: register adopted as Appendix A.19,
  IEC deviations recorded, earlier permit applications
- TP-CW1/CW2 need date moved to the EIA marine-works window; lesson L-EPCE-0002

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TuQPCZMPzEzscTVqEEHFMo
</commit_message>
<xml_diff>
--- a/output/clarification_register/ALP_clarification_register_ALP-CA-001.xlsx
+++ b/output/clarification_register/ALP_clarification_register_ALP-CA-001.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q25"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -481,7 +481,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>engine clarification_register v1.1.0 | generated 2026-09-28T03:43:27Z by SETUP | data 739c56375ca05fc7</t>
+          <t>engine clarification_register v1.1.0 | generated 2026-09-28T03:56:48Z by SETUP | data 86fb906a41f93ae0</t>
         </is>
       </c>
     </row>
@@ -2327,6 +2327,96 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>TQ-IEC-022</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Istanbul EPC</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Codes and standards back-to-back, and IEC deliverables for permits</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>The codes and standards register (Appendix A.19, proposed to the Owner in TQ-033) names IEC as responsible for 62 entries (power island design, tests, Turkish regulations applicable to the IEC supply). Please confirm compliance back-to-back and state any deviation, in particular: (1) ER-06.02 allows ASME Section I or EN 12952 - which code, which PED module; ER-06.05 cites EN 12952-3 for the cyclic assessment; (2) HEI edition for the condenser (ER-07.07: 11th or later); (3) GT enclosure fire protection (ER-10.05: water mist or CO2); (4) IEC 62443 SL2 for the TCS. (5) Confirm the IEC deliverables for the permits PMT-004, 005, 008, 009, 013, 014, 015, 016, 018 and 021 with the dates of the permits register.</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>ASME Section I with PED module G; EN 12952-3 for fatigue of thick-walled parts; HEI 12th edition; CO2 per NFPA 12; SL2; IEC deliverables 30 days before each apply-by date.</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>reference:REF-CONS-0042
+reference:REF-CONS-0043
+reference:REF-CONS-0045
+reference:REF-CONS-0082
+requirement:ER-06.02
+requirement:ER-06.05
+requirement:ER-07.07
+requirement:ER-10.05
+permit:PMT-004
+permit:PMT-015</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed back-to-back for all entries naming IEC, with: (1) HRSG to ASME Section I, PED module G by a notified body; EN 12952-3 for the low-cycle fatigue of the HP drum and SH/RH outlet headers; (2) HEI 12th edition; (3) GT enclosure CO2 total flooding per NFPA 12; (4) TCS system SL2 (IEC 62443-3-3) with certified components; please add ISO 20816-2 for the vibration limits of the turbines and generators. (5) IEC deliverables for the permits 30 days before each apply-by date of the permits register: generator/GSU data and models (PMT-004, PMT-021), foundation loads (PMT-005), heavy piece list and transport drawings (PMT-008, PMT-009), NDT source licences of IEC's site subcontractors (PMT-013), GT gas demand (PMT-014), inventories (PMT-015), declarations of conformity and notified body certificates (PMT-016), GT emission data (PMT-018).</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>contractor proposal accepted</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>technical_only</t>
+        </is>
+      </c>
+      <c r="P26" s="4" t="n"/>
+      <c r="Q26" s="5" t="inlineStr">
+        <is>
+          <t>reference/REF-CONS-0043
+reference/REF-CONS-0042
+reference/REF-CONS-0045
+reference/REF-CONS-0048
+reference/REF-CONS-0082</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:Q4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2479,10 +2569,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -2498,10 +2588,10 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>0</v>
@@ -2543,7 +2633,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">

</xml_diff>